<commit_message>
hdfc by razor pay payment gateway
</commit_message>
<xml_diff>
--- a/SMEnterprise/Content/Uploads/StudentList-Upload.xlsx
+++ b/SMEnterprise/Content/Uploads/StudentList-Upload.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="75">
   <si>
     <t>S.No.</t>
   </si>
@@ -67,143 +67,637 @@
     <t>DOJ</t>
   </si>
   <si>
-    <t xml:space="preserve">RAM CHANDRA </t>
-  </si>
-  <si>
-    <t>BHAWANI SHANKAR</t>
-  </si>
-  <si>
-    <t>SEEMA DEVI</t>
-  </si>
-  <si>
-    <t>TENUDARD</t>
-  </si>
-  <si>
-    <t>CHHAPWA</t>
-  </si>
-  <si>
-    <t>DEWARIYA</t>
-  </si>
-  <si>
-    <t>BASHIYA</t>
-  </si>
-  <si>
-    <t>LOUKHI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VIMLESH YADAV </t>
-  </si>
-  <si>
-    <t xml:space="preserve">RAM SUMER YADAV </t>
-  </si>
-  <si>
-    <t xml:space="preserve">VINDRAWATI DEVI </t>
-  </si>
-  <si>
-    <t>MATHIYPAR</t>
-  </si>
-  <si>
-    <t>RANDHEER SINGH</t>
-  </si>
-  <si>
-    <t>SADHANA</t>
-  </si>
-  <si>
-    <t>ANURADHA YADAV</t>
-  </si>
-  <si>
-    <t>24/8/2010</t>
-  </si>
-  <si>
-    <t>EKTASINGH</t>
-  </si>
-  <si>
-    <t>DEWRIYA</t>
-  </si>
-  <si>
-    <t>PRIYA</t>
-  </si>
-  <si>
-    <t>REETA YADAV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RAMBHA CHORSIYA </t>
-  </si>
-  <si>
-    <t>UPENDRA CHOURSIYA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MANJU </t>
-  </si>
-  <si>
-    <t>SHERYA CHOUDHARY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SHRADDHA  PANDAY  </t>
-  </si>
-  <si>
-    <t>ARVIND PANDAY</t>
-  </si>
-  <si>
-    <t>HARSITA</t>
-  </si>
-  <si>
-    <t>19/3/2013</t>
-  </si>
-  <si>
-    <t>DHEERAJ NISHAD</t>
-  </si>
-  <si>
-    <t>RAM SUBHAGE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ANEETA DEVI </t>
-  </si>
-  <si>
-    <t xml:space="preserve">KRISHNA TIWARI </t>
-  </si>
-  <si>
-    <t>SANTOSH TIWARI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NADANI TIWARI </t>
-  </si>
-  <si>
-    <t>NITIN YADAV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SUMITA DEVI </t>
-  </si>
-  <si>
-    <t xml:space="preserve">RAJAN CHOUDHARY </t>
-  </si>
-  <si>
-    <t>CHHOTELAL CHOUDHARY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BHANMATI DEVI </t>
-  </si>
-  <si>
-    <t>21/10/2009</t>
-  </si>
-  <si>
-    <t>NIDHI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SURENDRA </t>
-  </si>
-  <si>
-    <t xml:space="preserve">KHUSHI </t>
-  </si>
-  <si>
-    <t xml:space="preserve">LALJI GOUTAM </t>
+    <t xml:space="preserve">Naguran </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hasanpur </t>
+  </si>
+  <si>
+    <t>Naguran</t>
+  </si>
+  <si>
+    <t>Raichandwala</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mohangarh </t>
+  </si>
+  <si>
+    <t>Bhonsla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amerheri </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dhankheri </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Priya</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mr. Sanjay</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mrs. Reena</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Preeti</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mr. Rajkamal</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mrs. Santosh</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Yash</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mrs. Meena</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Aditya</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mr. Mahabeer</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mrs. Poonam</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Hitu</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mr. Surender</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Ankush</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mr. Ramesh</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mrs. Kamlesh</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Aryan
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Vansh</t>
+    </r>
+  </si>
+  <si>
+    <t>0
+0</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Mr. Rameher
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mr. Bijender</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">8685067534
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>7988303326</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Mrs. koshalya
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mrs. Meena</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Kartik</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mr.Umed</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mrs. Kiran</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Arun</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mr.Manoj</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Arman</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mr. Joginder</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mrs. Asha</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Lakshya</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mr. Radheshyam</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Harshit</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mr. Sandeep</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mrs. Suman</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Tamanna</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mr. Jagbir</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mrs. Renu</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Nitesh
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Lakshya</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Mr. kaptan
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mr.Ramdiya</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">8053384266
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>8708171984</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Mrs. Sunita
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mrs. Saroj</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Parveen</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mr.Birender</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Uttam
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Shourya</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Mr.Gurudev
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mr.Sukhvinder</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">9729590705
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>9896010616</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Mrs. Bhateri
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mrs. Suman</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Abhishekh</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mr.Balkar</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mrs. Rekha</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="3">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -226,6 +720,26 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="9.5"/>
+      <name val="Arial MT"/>
+    </font>
+    <font>
+      <sz val="9.5"/>
+      <name val="Arial MT"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9.5"/>
+      <color rgb="FF000000"/>
+      <name val="Arial MT"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -240,7 +754,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -263,12 +777,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -284,8 +813,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" shrinkToFit="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1415,7 +1952,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q34"/>
+  <dimension ref="A1:Q19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
@@ -1489,413 +2026,568 @@
       </c>
     </row>
     <row r="2" spans="1:17">
-      <c r="A2" s="6">
+      <c r="A2" s="9">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>153</v>
-      </c>
-      <c r="C2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D2">
-        <v>207</v>
-      </c>
-      <c r="F2">
+      <c r="B2" s="7"/>
+      <c r="C2" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="10">
         <v>1</v>
       </c>
-      <c r="G2" t="s">
-        <v>25</v>
-      </c>
-      <c r="H2">
-        <v>7408716752</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>28</v>
+      <c r="G2" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="H2" s="11">
+        <v>7015741025</v>
+      </c>
+      <c r="I2" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="J2" s="7"/>
+      <c r="K2" s="7"/>
+      <c r="L2" s="7"/>
+      <c r="M2" s="7"/>
+      <c r="N2" s="7"/>
+      <c r="O2" s="7"/>
+      <c r="P2" s="7"/>
+      <c r="Q2" s="9" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:17">
-      <c r="A3" s="6">
+      <c r="A3" s="9">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>327</v>
-      </c>
-      <c r="C3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D3">
-        <v>208</v>
-      </c>
-      <c r="F3">
+      <c r="B3" s="7"/>
+      <c r="C3" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="10">
         <v>1</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="I3" t="s">
+      <c r="H3" s="11">
+        <v>8529705213</v>
+      </c>
+      <c r="I3" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="Q3" t="s">
-        <v>34</v>
+      <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
+      <c r="O3" s="7"/>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="9" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:17">
-      <c r="A4" s="6">
+      <c r="A4" s="9">
         <v>3</v>
       </c>
-      <c r="B4">
-        <v>344</v>
-      </c>
-      <c r="C4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D4">
-        <v>209</v>
-      </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="G4" t="s">
-        <v>17</v>
-      </c>
-      <c r="H4">
-        <v>9888365895</v>
-      </c>
-      <c r="I4" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>28</v>
+      <c r="B4" s="7"/>
+      <c r="C4" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="10">
+        <v>0</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" s="11">
+        <v>9416107612</v>
+      </c>
+      <c r="I4" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="7"/>
+      <c r="M4" s="7"/>
+      <c r="N4" s="7"/>
+      <c r="O4" s="7"/>
+      <c r="P4" s="7"/>
+      <c r="Q4" s="9" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:17">
-      <c r="A5" s="6">
+      <c r="A5" s="9">
         <v>4</v>
       </c>
-      <c r="B5">
-        <v>279</v>
-      </c>
-      <c r="C5" t="s">
-        <v>37</v>
-      </c>
-      <c r="D5">
-        <v>210</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-      <c r="G5" t="s">
-        <v>38</v>
-      </c>
-      <c r="H5">
-        <v>8948331006</v>
-      </c>
-      <c r="I5" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>28</v>
+      <c r="B5" s="7"/>
+      <c r="C5" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="10">
+        <v>0</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="H5" s="11">
+        <v>9255182120</v>
+      </c>
+      <c r="I5" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="7"/>
+      <c r="P5" s="7"/>
+      <c r="Q5" s="9" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:17">
-      <c r="A6" s="6">
+      <c r="A6" s="9">
         <v>5</v>
       </c>
-      <c r="B6">
-        <v>366</v>
-      </c>
-      <c r="C6" t="s">
-        <v>40</v>
-      </c>
-      <c r="D6">
-        <v>211</v>
-      </c>
-      <c r="F6">
-        <v>1</v>
-      </c>
-      <c r="G6" t="s">
-        <v>18</v>
-      </c>
-      <c r="H6">
-        <v>9792772055</v>
-      </c>
-      <c r="I6" t="s">
+      <c r="B6" s="7"/>
+      <c r="C6" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="10">
+        <v>0</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="H6" s="11">
+        <v>8529210000</v>
+      </c>
+      <c r="I6" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7"/>
+      <c r="L6" s="7"/>
+      <c r="M6" s="7"/>
+      <c r="N6" s="7"/>
+      <c r="O6" s="7"/>
+      <c r="P6" s="7"/>
+      <c r="Q6" s="9" t="s">
         <v>19</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:17">
-      <c r="A7" s="6">
+      <c r="A7" s="9">
         <v>6</v>
       </c>
-      <c r="B7">
-        <v>285</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="B7" s="7"/>
+      <c r="C7" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="10">
+        <v>0</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="H7" s="11">
+        <v>7206461949</v>
+      </c>
+      <c r="I7" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="7"/>
+      <c r="N7" s="7"/>
+      <c r="O7" s="7"/>
+      <c r="P7" s="7"/>
+      <c r="Q7" s="9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" ht="30">
+      <c r="A8" s="9">
+        <v>7</v>
+      </c>
+      <c r="B8" s="7"/>
+      <c r="C8" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="D7">
-        <v>212</v>
-      </c>
-      <c r="F7">
-        <v>1</v>
-      </c>
-      <c r="G7" t="s">
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="H7">
-        <v>9792566355</v>
-      </c>
-      <c r="I7" t="s">
+      <c r="G8" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="K7" s="4" t="s">
+      <c r="H8" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="Q7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17">
-      <c r="A8" s="6">
-        <v>7</v>
-      </c>
-      <c r="B8">
-        <v>377</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="I8" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="D8">
-        <v>213</v>
-      </c>
-      <c r="F8">
-        <v>0</v>
-      </c>
-      <c r="G8" t="s">
-        <v>46</v>
-      </c>
-      <c r="H8">
-        <v>9838340349</v>
-      </c>
-      <c r="I8" t="s">
-        <v>47</v>
-      </c>
-      <c r="K8" s="4">
-        <v>40179</v>
-      </c>
-      <c r="Q8" t="s">
-        <v>22</v>
+      <c r="J8" s="7"/>
+      <c r="K8" s="7"/>
+      <c r="L8" s="7"/>
+      <c r="M8" s="7"/>
+      <c r="N8" s="7"/>
+      <c r="O8" s="7"/>
+      <c r="P8" s="7"/>
+      <c r="Q8" s="9" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:17">
-      <c r="A9" s="6">
+      <c r="A9" s="9">
         <v>8</v>
       </c>
-      <c r="B9">
-        <v>223</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="B9" s="7"/>
+      <c r="C9" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="10">
+        <v>0</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="H9" s="11">
+        <v>9468153026</v>
+      </c>
+      <c r="I9" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="D9">
-        <v>214</v>
-      </c>
-      <c r="F9">
-        <v>0</v>
-      </c>
-      <c r="G9" t="s">
-        <v>49</v>
-      </c>
-      <c r="H9">
-        <v>9554945471</v>
-      </c>
-      <c r="I9" t="s">
-        <v>50</v>
-      </c>
-      <c r="Q9" t="s">
-        <v>21</v>
+      <c r="J9" s="7"/>
+      <c r="K9" s="7"/>
+      <c r="L9" s="7"/>
+      <c r="M9" s="7"/>
+      <c r="N9" s="7"/>
+      <c r="O9" s="7"/>
+      <c r="P9" s="7"/>
+      <c r="Q9" s="9" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:17">
-      <c r="A10" s="6">
+      <c r="A10" s="9">
         <v>9</v>
       </c>
-      <c r="B10">
-        <v>177</v>
-      </c>
-      <c r="C10" t="s">
-        <v>51</v>
-      </c>
-      <c r="D10">
-        <v>215</v>
-      </c>
-      <c r="F10">
+      <c r="B10" s="7"/>
+      <c r="C10" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="10">
         <v>0</v>
       </c>
-      <c r="G10" t="s">
-        <v>26</v>
-      </c>
-      <c r="H10">
-        <v>9167033980</v>
-      </c>
-      <c r="I10" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q10" t="s">
+      <c r="G10" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="H10" s="11">
+        <v>9588524512</v>
+      </c>
+      <c r="I10" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="7"/>
+      <c r="N10" s="7"/>
+      <c r="O10" s="7"/>
+      <c r="P10" s="7"/>
+      <c r="Q10" s="9" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:17">
-      <c r="A11" s="6">
+      <c r="A11" s="9">
         <v>10</v>
       </c>
-      <c r="B11">
-        <v>341</v>
-      </c>
-      <c r="C11" t="s">
+      <c r="B11" s="7"/>
+      <c r="C11" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="10">
+        <v>0</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H11" s="11">
+        <v>9812866058</v>
+      </c>
+      <c r="I11" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="D11">
-        <v>216</v>
-      </c>
-      <c r="F11">
-        <v>0</v>
-      </c>
-      <c r="G11" t="s">
-        <v>54</v>
-      </c>
-      <c r="H11">
-        <v>6307397031</v>
-      </c>
-      <c r="I11" t="s">
-        <v>55</v>
-      </c>
-      <c r="K11" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="Q11" t="s">
-        <v>28</v>
+      <c r="J11" s="7"/>
+      <c r="K11" s="7"/>
+      <c r="L11" s="7"/>
+      <c r="M11" s="7"/>
+      <c r="N11" s="7"/>
+      <c r="O11" s="7"/>
+      <c r="P11" s="7"/>
+      <c r="Q11" s="9" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:17">
-      <c r="A12" s="6">
+      <c r="A12" s="9">
         <v>11</v>
       </c>
-      <c r="C12" t="s">
-        <v>57</v>
-      </c>
-      <c r="D12">
-        <v>217</v>
-      </c>
-      <c r="F12">
-        <v>1</v>
-      </c>
-      <c r="G12" t="s">
-        <v>58</v>
-      </c>
-      <c r="I12" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q12" t="s">
-        <v>24</v>
+      <c r="B12" s="7"/>
+      <c r="C12" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="10">
+        <v>0</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="H12" s="11">
+        <v>9966820739</v>
+      </c>
+      <c r="I12" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="J12" s="7"/>
+      <c r="K12" s="7"/>
+      <c r="L12" s="7"/>
+      <c r="M12" s="7"/>
+      <c r="N12" s="7"/>
+      <c r="O12" s="7"/>
+      <c r="P12" s="7"/>
+      <c r="Q12" s="9" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:17">
-      <c r="A13" s="6">
+      <c r="A13" s="9">
         <v>12</v>
       </c>
-      <c r="C13" t="s">
-        <v>59</v>
-      </c>
-      <c r="D13">
-        <v>218</v>
-      </c>
-      <c r="F13">
-        <v>1</v>
-      </c>
-      <c r="G13" t="s">
-        <v>60</v>
-      </c>
-      <c r="H13">
-        <v>9565308211</v>
-      </c>
-      <c r="I13" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q13" t="s">
-        <v>23</v>
+      <c r="B13" s="7"/>
+      <c r="C13" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="10">
+        <v>0</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="H13" s="11">
+        <v>9253556556</v>
+      </c>
+      <c r="I13" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="J13" s="7"/>
+      <c r="K13" s="7"/>
+      <c r="L13" s="7"/>
+      <c r="M13" s="7"/>
+      <c r="N13" s="7"/>
+      <c r="O13" s="7"/>
+      <c r="P13" s="7"/>
+      <c r="Q13" s="9" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:17">
-      <c r="A14" s="6"/>
+      <c r="A14" s="9">
+        <v>13</v>
+      </c>
+      <c r="B14" s="7"/>
+      <c r="C14" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="10">
+        <v>1</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="H14" s="11">
+        <v>9812310874</v>
+      </c>
+      <c r="I14" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="J14" s="7"/>
+      <c r="K14" s="7"/>
+      <c r="L14" s="7"/>
+      <c r="M14" s="7"/>
+      <c r="N14" s="7"/>
+      <c r="O14" s="7"/>
+      <c r="P14" s="7"/>
+      <c r="Q14" s="9" t="s">
+        <v>19</v>
+      </c>
     </row>
-    <row r="15" spans="1:17">
-      <c r="A15" s="6"/>
+    <row r="15" spans="1:17" ht="30">
+      <c r="A15" s="9">
+        <v>14</v>
+      </c>
+      <c r="B15" s="7"/>
+      <c r="C15" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="H15" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="I15" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="J15" s="7"/>
+      <c r="K15" s="7"/>
+      <c r="L15" s="7"/>
+      <c r="M15" s="7"/>
+      <c r="N15" s="7"/>
+      <c r="O15" s="7"/>
+      <c r="P15" s="7"/>
+      <c r="Q15" s="9" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="16" spans="1:17">
-      <c r="A16" s="6"/>
+      <c r="A16" s="9">
+        <v>15</v>
+      </c>
+      <c r="B16" s="7"/>
+      <c r="C16" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="10">
+        <v>0</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="H16" s="11">
+        <v>9728079421</v>
+      </c>
+      <c r="I16" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="J16" s="7"/>
+      <c r="K16" s="7"/>
+      <c r="L16" s="7"/>
+      <c r="M16" s="7"/>
+      <c r="N16" s="7"/>
+      <c r="O16" s="7"/>
+      <c r="P16" s="7"/>
+      <c r="Q16" s="9" t="s">
+        <v>23</v>
+      </c>
     </row>
-    <row r="17" spans="1:7">
-      <c r="A17" s="6"/>
+    <row r="17" spans="1:17" ht="30">
+      <c r="A17" s="9">
+        <v>16</v>
+      </c>
+      <c r="B17" s="7"/>
+      <c r="C17" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="G17" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="H17" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="I17" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="J17" s="7"/>
+      <c r="K17" s="7"/>
+      <c r="L17" s="7"/>
+      <c r="M17" s="7"/>
+      <c r="N17" s="7"/>
+      <c r="O17" s="7"/>
+      <c r="P17" s="7"/>
+      <c r="Q17" s="9" t="s">
+        <v>19</v>
+      </c>
     </row>
-    <row r="18" spans="1:7">
-      <c r="A18" s="6"/>
-      <c r="G18" s="7"/>
+    <row r="18" spans="1:17">
+      <c r="A18" s="9">
+        <v>17</v>
+      </c>
+      <c r="B18" s="7"/>
+      <c r="C18" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="10">
+        <v>0</v>
+      </c>
+      <c r="G18" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="H18" s="11">
+        <v>9499472285</v>
+      </c>
+      <c r="I18" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="J18" s="7"/>
+      <c r="K18" s="7"/>
+      <c r="L18" s="7"/>
+      <c r="M18" s="7"/>
+      <c r="N18" s="7"/>
+      <c r="O18" s="7"/>
+      <c r="P18" s="7"/>
+      <c r="Q18" s="9" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="19" spans="1:7">
+    <row r="19" spans="1:17">
       <c r="A19" s="6"/>
-    </row>
-    <row r="20" spans="1:7">
-      <c r="A20" s="6"/>
-    </row>
-    <row r="21" spans="1:7">
-      <c r="A21" s="6"/>
-    </row>
-    <row r="22" spans="1:7">
-      <c r="A22" s="6"/>
-    </row>
-    <row r="23" spans="1:7">
-      <c r="A23" s="6"/>
-    </row>
-    <row r="24" spans="1:7">
-      <c r="A24" s="6"/>
-    </row>
-    <row r="25" spans="1:7">
-      <c r="A25" s="6"/>
-    </row>
-    <row r="26" spans="1:7">
-      <c r="A26" s="6"/>
-    </row>
-    <row r="27" spans="1:7">
-      <c r="A27" s="6"/>
-    </row>
-    <row r="28" spans="1:7">
-      <c r="A28" s="6"/>
-    </row>
-    <row r="29" spans="1:7">
-      <c r="A29" s="6"/>
-    </row>
-    <row r="30" spans="1:7">
-      <c r="A30" s="6"/>
-    </row>
-    <row r="31" spans="1:7">
-      <c r="A31" s="6"/>
-    </row>
-    <row r="32" spans="1:7">
-      <c r="A32" s="6"/>
-    </row>
-    <row r="33" spans="1:1">
-      <c r="A33" s="6"/>
-    </row>
-    <row r="34" spans="1:1">
-      <c r="A34" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>